<commit_message>
Update git search to include multi_dot
</commit_message>
<xml_diff>
--- a/SearchGit/Results/Summary_Top_100.xlsx
+++ b/SearchGit/Results/Summary_Top_100.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,11 @@
           <t>matmul</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>multi_dot</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -465,6 +470,9 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +489,9 @@
       <c r="D3" t="n">
         <v>0</v>
       </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -497,6 +508,9 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -513,6 +527,9 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -529,6 +546,9 @@
       <c r="D6" t="n">
         <v>15</v>
       </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -545,11 +565,14 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>yt-dlp/yt-dlp</t>
+          <t>NousResearch/hermes-agent</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -559,38 +582,47 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUTOMATIC1111/stable-diffusion-webui</t>
+          <t>yt-dlp/yt-dlp</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NousResearch/hermes-agent</t>
+          <t>AUTOMATIC1111/stable-diffusion-webui</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -607,7 +639,10 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>375</v>
+        <v>374</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -625,6 +660,9 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -641,11 +679,14 @@
       <c r="D13" t="n">
         <v>0</v>
       </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ytdl-org/youtube-dl</t>
+          <t>anthropics/skills</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -655,13 +696,16 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>anthropics/skills</t>
+          <t>ytdl-org/youtube-dl</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -671,6 +715,9 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -689,6 +736,9 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -705,6 +755,9 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -721,85 +774,103 @@
       <c r="D18" t="n">
         <v>0</v>
       </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Comfy-Org/ComfyUI</t>
+          <t>anthropics/claude-code</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>78</v>
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shubhamsaboo/awesome-llm-apps</t>
+          <t>Comfy-Org/ComfyUI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
+        <v>93</v>
+      </c>
+      <c r="E20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>github/spec-kit</t>
+          <t>Shubhamsaboo/awesome-llm-apps</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>deepseek-ai/DeepSeek-V3</t>
+          <t>github/spec-kit</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>pytorch/pytorch</t>
+          <t>deepseek-ai/DeepSeek-V3</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>164</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>981</v>
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -817,27 +888,33 @@
       <c r="D24" t="n">
         <v>4</v>
       </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>fastapi/fastapi</t>
+          <t>pytorch/pytorch</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>981</v>
+      </c>
+      <c r="E25" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>nvbn/thefuck</t>
+          <t>fastapi/fastapi</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -847,13 +924,16 @@
         <v>0</v>
       </c>
       <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>browser-use/browser-use</t>
+          <t>nvbn/thefuck</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -863,45 +943,54 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>hacksider/Deep-Live-Cam</t>
+          <t>browser-use/browser-use</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>django/django</t>
+          <t>hacksider/Deep-Live-Cam</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>home-assistant/core</t>
+          <t>django/django</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -911,45 +1000,54 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3b1b/manim</t>
+          <t>home-assistant/core</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sherlock-project/sherlock</t>
+          <t>3b1b/manim</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>karpathy/autoresearch</t>
+          <t>nextlevelbuilder/ui-ux-pro-max-skill</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -959,13 +1057,16 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>bregman-arie/devops-exercises</t>
+          <t>karpathy/autoresearch</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -975,13 +1076,16 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>nextlevelbuilder/ui-ux-pro-max-skill</t>
+          <t>sherlock-project/sherlock</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -991,38 +1095,47 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>infiniflow/ragflow</t>
+          <t>bregman-arie/devops-exercises</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>fighting41love/funNLP</t>
+          <t>infiniflow/ragflow</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1033,35 +1146,41 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>125</v>
+        <v>127</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PaddlePaddle/PaddleOCR</t>
+          <t>TauricResearch/TradingAgents</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TauricResearch/TradingAgents</t>
+          <t>fighting41love/funNLP</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1071,22 +1190,28 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>d2l-ai/d2l-zh</t>
+          <t>PaddlePaddle/PaddleOCR</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
       </c>
       <c r="D41" t="n">
+        <v>10</v>
+      </c>
+      <c r="E41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1105,43 +1230,52 @@
       <c r="D42" t="n">
         <v>0</v>
       </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>tensorflow/models</t>
+          <t>d2l-ai/d2l-zh</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Z4nzu/hackingtool</t>
+          <t>tensorflow/models</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OpenHands/OpenHands</t>
+          <t>Z4nzu/hackingtool</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1151,29 +1285,35 @@
         <v>0</v>
       </c>
       <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>python/cpython</t>
+          <t>OpenHands/OpenHands</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>josephmisiti/awesome-machine-learning</t>
+          <t>harry0703/MoneyPrinterTurbo</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1183,61 +1323,73 @@
         <v>0</v>
       </c>
       <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>pallets/flask</t>
+          <t>python/cpython</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
+        <v>15</v>
+      </c>
+      <c r="E48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>hiyouga/LlamaFactory</t>
+          <t>josephmisiti/awesome-machine-learning</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>binary-husky/gpt_academic</t>
+          <t>hiyouga/LlamaFactory</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
       <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>bytedance/deer-flow</t>
+          <t>pallets/flask</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1247,13 +1399,16 @@
         <v>0</v>
       </c>
       <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ansible/ansible</t>
+          <t>binary-husky/gpt_academic</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1263,29 +1418,35 @@
         <v>0</v>
       </c>
       <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>FoundationAgents/MetaGPT</t>
+          <t>bytedance/deer-flow</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C53" t="n">
         <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OpenBB-finance/OpenBB</t>
+          <t>ansible/ansible</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1295,29 +1456,35 @@
         <v>0</v>
       </c>
       <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>labmlai/annotated_deep_learning_paper_implementations</t>
+          <t>FoundationAgents/MetaGPT</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C55" t="n">
         <v>0</v>
       </c>
       <c r="D55" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>xtekky/gpt4free</t>
+          <t>OpenBB-finance/OpenBB</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1327,45 +1494,54 @@
         <v>0</v>
       </c>
       <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>scikit-learn/scikit-learn</t>
+          <t>unclecode/crawl4ai</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>547</v>
+        <v>7</v>
       </c>
       <c r="C57" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>319</v>
+        <v>2</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>unclecode/crawl4ai</t>
+          <t>labmlai/annotated_deep_learning_paper_implementations</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>localstack/localstack</t>
+          <t>xtekky/gpt4free</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1375,23 +1551,29 @@
         <v>0</v>
       </c>
       <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>unslothai/unsloth</t>
+          <t>scikit-learn/scikit-learn</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
+        <v>547</v>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="D60" t="n">
-        <v>24</v>
+        <v>319</v>
+      </c>
+      <c r="E60" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="61">
@@ -1409,27 +1591,33 @@
       <c r="D61" t="n">
         <v>1</v>
       </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>keras-team/keras</t>
+          <t>unslothai/unsloth</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="C62" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>openinterpreter/open-interpreter</t>
+          <t>localstack/localstack</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1439,29 +1627,35 @@
         <v>0</v>
       </c>
       <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>pathwaycom/pathway</t>
+          <t>keras-team/keras</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D64" t="n">
-        <v>7</v>
+        <v>22</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Asabeneh/30-Days-Of-Python</t>
+          <t>shareAI-lab/learn-claude-code</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1471,13 +1665,16 @@
         <v>0</v>
       </c>
       <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>shareAI-lab/learn-claude-code</t>
+          <t>openinterpreter/open-interpreter</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1487,13 +1684,16 @@
         <v>0</v>
       </c>
       <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>scrapy/scrapy</t>
+          <t>Asabeneh/30-Days-Of-Python</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1503,6 +1703,9 @@
         <v>0</v>
       </c>
       <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1521,43 +1724,52 @@
       <c r="D68" t="n">
         <v>0</v>
       </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ComposioHQ/awesome-claude-skills</t>
+          <t>pathwaycom/pathway</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
+        <v>7</v>
+      </c>
+      <c r="E69" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>commaai/openpilot</t>
+          <t>ComposioHQ/awesome-claude-skills</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>48</v>
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>docling-project/docling</t>
+          <t>scrapy/scrapy</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1567,29 +1779,35 @@
         <v>0</v>
       </c>
       <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CorentinJ/Real-Time-Voice-Cloning</t>
+          <t>commaai/openpilot</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D72" t="n">
-        <v>1</v>
+        <v>48</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>meta-llama/llama</t>
+          <t>docling-project/docling</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1599,29 +1817,35 @@
         <v>0</v>
       </c>
       <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>virattt/ai-hedge-fund</t>
+          <t>CorentinJ/Real-Time-Voice-Cloning</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
       </c>
       <c r="D74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>karpathy/nanoGPT</t>
+          <t>virattt/ai-hedge-fund</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1631,13 +1855,16 @@
         <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>microsoft/autogen</t>
+          <t>meta-llama/llama</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1647,13 +1874,16 @@
         <v>0</v>
       </c>
       <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sansan0/TrendRadar</t>
+          <t>karpathy/nanoGPT</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1663,13 +1893,16 @@
         <v>0</v>
       </c>
       <c r="D77" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>RVC-Boss/GPT-SoVITS</t>
+          <t>sansan0/TrendRadar</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1679,13 +1912,16 @@
         <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>harry0703/MoneyPrinterTurbo</t>
+          <t>microsoft/autogen</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1695,45 +1931,54 @@
         <v>0</v>
       </c>
       <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ultralytics/ultralytics</t>
+          <t>RVC-Boss/GPT-SoVITS</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
       </c>
       <c r="D80" t="n">
-        <v>33</v>
+        <v>5</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ultralytics/yolov5</t>
+          <t>ultralytics/ultralytics</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="E81" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>zylon-ai/private-gpt</t>
+          <t>safishamsi/graphify</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1743,13 +1988,16 @@
         <v>0</v>
       </c>
       <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>soimort/you-get</t>
+          <t>ultralytics/yolov5</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1759,29 +2007,35 @@
         <v>0</v>
       </c>
       <c r="D83" t="n">
+        <v>15</v>
+      </c>
+      <c r="E83" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Textualize/rich</t>
+          <t>mem0ai/mem0</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
       </c>
       <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ageitgey/face_recognition</t>
+          <t>zylon-ai/private-gpt</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1791,29 +2045,35 @@
         <v>0</v>
       </c>
       <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>mem0ai/mem0</t>
+          <t>D4Vinci/Scrapling</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FoundationAgents/OpenManus</t>
+          <t>soimort/you-get</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1823,29 +2083,35 @@
         <v>0</v>
       </c>
       <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>deepfakes/faceswap</t>
+          <t>Textualize/rich</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>26</v>
+        <v>0</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>AntonOsika/gpt-engineer</t>
+          <t>FoundationAgents/OpenManus</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1855,13 +2121,16 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Zie619/n8n-workflows</t>
+          <t>ageitgey/face_recognition</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1871,29 +2140,35 @@
         <v>0</v>
       </c>
       <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>psf/requests</t>
+          <t>deepfakes/faceswap</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C91" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D91" t="n">
+        <v>26</v>
+      </c>
+      <c r="E91" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>karpathy/nanochat</t>
+          <t>AntonOsika/gpt-engineer</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1903,29 +2178,35 @@
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>D4Vinci/Scrapling</t>
+          <t>datawhalechina/hello-agents</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C93" t="n">
         <v>0</v>
       </c>
       <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MemPalace/mempalace</t>
+          <t>Zie619/n8n-workflows</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1935,29 +2216,35 @@
         <v>0</v>
       </c>
       <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>datawhalechina/hello-agents</t>
+          <t>karpathy/nanochat</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C95" t="n">
         <v>0</v>
       </c>
       <c r="D95" t="n">
+        <v>6</v>
+      </c>
+      <c r="E95" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>crewAIInc/crewAI</t>
+          <t>psf/requests</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1967,29 +2254,35 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>xai-org/grok-1</t>
+          <t>MemPalace/mempalace</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
         <v>0</v>
       </c>
       <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>charlax/professional-programming</t>
+          <t>crewAIInc/crewAI</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1999,6 +2292,9 @@
         <v>0</v>
       </c>
       <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2017,27 +2313,33 @@
       <c r="D99" t="n">
         <v>0</v>
       </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>safishamsi/graphify</t>
+          <t>xai-org/grok-1</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C100" t="n">
         <v>0</v>
       </c>
       <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>freqtrade/freqtrade</t>
+          <t>charlax/professional-programming</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2047,6 +2349,9 @@
         <v>0</v>
       </c>
       <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>